<commit_message>
feat(ui): remove 'all years + future' filter, wage KPI card, and MoM volatility chart from homepage
</commit_message>
<xml_diff>
--- a/gold.xlsx
+++ b/gold.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hamahang\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hamahang\Desktop\روند رشد طلا\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A42C1B-3F97-4C22-856C-0ACDECAFA2FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D4DA4A-774E-4689-AE84-3C92E12FC69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="جدول اصلی" sheetId="1" r:id="rId1"/>
     <sheet name="نسبت خقوق پایه به قیمت طلا" sheetId="4" r:id="rId2"/>
-    <sheet name="نمودار رشد" sheetId="2" r:id="rId3"/>
-    <sheet name="میانگین طلا در ماه" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId3"/>
+    <sheet name="نمودار رشد" sheetId="2" r:id="rId4"/>
+    <sheet name="میانگین طلا در ماه" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -546,10 +547,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -728,7 +730,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -808,6 +810,11 @@
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -826,11 +833,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -4716,12 +4739,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
@@ -4734,40 +4757,40 @@
       <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="29">
+      <c r="D2" s="32">
         <v>1395</v>
       </c>
-      <c r="E2" s="29">
+      <c r="E2" s="32">
         <v>1396</v>
       </c>
-      <c r="F2" s="29">
+      <c r="F2" s="32">
         <v>1397</v>
       </c>
-      <c r="G2" s="29">
+      <c r="G2" s="32">
         <v>1398</v>
       </c>
-      <c r="H2" s="29">
+      <c r="H2" s="32">
         <v>1399</v>
       </c>
-      <c r="I2" s="29">
+      <c r="I2" s="32">
         <v>1400</v>
       </c>
-      <c r="J2" s="29">
+      <c r="J2" s="32">
         <v>1401</v>
       </c>
-      <c r="K2" s="29">
+      <c r="K2" s="32">
         <v>1402</v>
       </c>
-      <c r="L2" s="29">
+      <c r="L2" s="32">
         <v>1403</v>
       </c>
-      <c r="M2" s="29">
+      <c r="M2" s="32">
         <v>1404</v>
       </c>
-      <c r="N2" s="29">
+      <c r="N2" s="32">
         <v>1405</v>
       </c>
     </row>
@@ -4776,25 +4799,25 @@
         <v>4</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
       <c r="D4" s="10">
         <v>972000</v>
       </c>
@@ -4830,11 +4853,11 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
       <c r="D5" s="26">
         <f>D4/D6</f>
         <v>8.7668465283242654</v>
@@ -4884,8 +4907,8 @@
       <c r="A6" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="20">
         <f>SUM(D7:D18)/COUNTA(D7:D18)</f>
         <v>110872.25</v>
@@ -4935,11 +4958,11 @@
       <c r="A7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B7" s="30">
         <f>(SUM(D7:N7))/COUNTA(D7:N7)</f>
         <v>3263089.7272727271</v>
       </c>
-      <c r="C7" s="27"/>
+      <c r="C7" s="30"/>
       <c r="D7" s="10">
         <v>103500</v>
       </c>
@@ -4978,11 +5001,11 @@
       <c r="A8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="30">
         <f>(SUM(D8:N8))/COUNTA(D8:N8)</f>
         <v>3262795.4545454546</v>
       </c>
-      <c r="C8" s="27"/>
+      <c r="C8" s="30"/>
       <c r="D8" s="10">
         <v>105750</v>
       </c>
@@ -5021,11 +5044,11 @@
       <c r="A9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="27">
+      <c r="B9" s="30">
         <f>(SUM(D9:N9))/COUNTA(D9:N9)</f>
         <v>3048536.0909090908</v>
       </c>
-      <c r="C9" s="27"/>
+      <c r="C9" s="30"/>
       <c r="D9" s="11">
         <v>101617</v>
       </c>
@@ -5064,11 +5087,11 @@
       <c r="A10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="27">
+      <c r="B10" s="30">
         <f t="shared" ref="B10:B18" si="2">(SUM(D10:N10))/COUNTA(D10:N10)</f>
         <v>3201205.4545454546</v>
       </c>
-      <c r="C10" s="27"/>
+      <c r="C10" s="30"/>
       <c r="D10" s="12">
         <v>111700</v>
       </c>
@@ -5107,11 +5130,11 @@
       <c r="A11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="30">
         <f t="shared" si="2"/>
         <v>3314881.8181818184</v>
       </c>
-      <c r="C11" s="27"/>
+      <c r="C11" s="30"/>
       <c r="D11" s="10">
         <v>113000</v>
       </c>
@@ -5150,11 +5173,11 @@
       <c r="A12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="30">
         <f>(SUM(D12:N12))/COUNTA(D12:N12)</f>
         <v>3832193.9090909092</v>
       </c>
-      <c r="C12" s="27"/>
+      <c r="C12" s="30"/>
       <c r="D12" s="18">
         <v>114000</v>
       </c>
@@ -5193,11 +5216,11 @@
       <c r="A13" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="30">
         <f t="shared" si="2"/>
         <v>2195750</v>
       </c>
-      <c r="C13" s="27"/>
+      <c r="C13" s="30"/>
       <c r="D13" s="14">
         <v>110000</v>
       </c>
@@ -5234,11 +5257,11 @@
       <c r="A14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="27">
+      <c r="B14" s="30">
         <f t="shared" si="2"/>
         <v>2249340</v>
       </c>
-      <c r="C14" s="27"/>
+      <c r="C14" s="30"/>
       <c r="D14" s="10">
         <v>113400</v>
       </c>
@@ -5275,11 +5298,11 @@
       <c r="A15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="27">
+      <c r="B15" s="30">
         <f t="shared" si="2"/>
         <v>2476810</v>
       </c>
-      <c r="C15" s="27"/>
+      <c r="C15" s="30"/>
       <c r="D15" s="10">
         <v>113500</v>
       </c>
@@ -5316,11 +5339,11 @@
       <c r="A16" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="27">
+      <c r="B16" s="30">
         <f t="shared" si="2"/>
         <v>2825890</v>
       </c>
-      <c r="C16" s="27"/>
+      <c r="C16" s="30"/>
       <c r="D16" s="10">
         <v>113000</v>
       </c>
@@ -5357,11 +5380,11 @@
       <c r="A17" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="30">
         <f t="shared" si="2"/>
         <v>3361960</v>
       </c>
-      <c r="C17" s="27"/>
+      <c r="C17" s="30"/>
       <c r="D17" s="10">
         <v>115000</v>
       </c>
@@ -5398,11 +5421,11 @@
       <c r="A18" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="30">
         <f t="shared" si="2"/>
         <v>3547100</v>
       </c>
-      <c r="C18" s="27"/>
+      <c r="C18" s="30"/>
       <c r="D18" s="13">
         <v>116000</v>
       </c>
@@ -5481,10 +5504,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="27" t="s">
         <v>154</v>
       </c>
     </row>
@@ -5492,7 +5515,7 @@
       <c r="A3" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="B3" s="34">
+      <c r="B3" s="28">
         <v>8.7668465283242654</v>
       </c>
     </row>
@@ -5500,7 +5523,7 @@
       <c r="A4" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="B4" s="34">
+      <c r="B4" s="28">
         <v>8.5647614257948685</v>
       </c>
     </row>
@@ -5508,7 +5531,7 @@
       <c r="A5" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="B5" s="34">
+      <c r="B5" s="28">
         <v>3.9897172236503855</v>
       </c>
     </row>
@@ -5516,7 +5539,7 @@
       <c r="A6" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="B6" s="34">
+      <c r="B6" s="28">
         <v>3.9786332657948056</v>
       </c>
     </row>
@@ -5524,7 +5547,7 @@
       <c r="A7" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="B7" s="34">
+      <c r="B7" s="28">
         <v>2.3752577319587629</v>
       </c>
     </row>
@@ -5532,7 +5555,7 @@
       <c r="A8" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="34">
+      <c r="B8" s="28">
         <v>3.2449024336768253</v>
       </c>
     </row>
@@ -5540,7 +5563,7 @@
       <c r="A9" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="34">
+      <c r="B9" s="28">
         <v>3.5801811401172081</v>
       </c>
     </row>
@@ -5548,7 +5571,7 @@
       <c r="A10" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="34">
+      <c r="B10" s="28">
         <v>2.7374631268436578</v>
       </c>
     </row>
@@ -5556,7 +5579,7 @@
       <c r="A11" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="34">
+      <c r="B11" s="28">
         <v>2.2381216501880754</v>
       </c>
     </row>
@@ -5564,7 +5587,7 @@
       <c r="A12" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="B12" s="34">
+      <c r="B12" s="28">
         <v>1.210743329140574</v>
       </c>
     </row>
@@ -5572,7 +5595,7 @@
       <c r="A13" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="28">
         <v>1.1651410968214599</v>
       </c>
     </row>
@@ -5584,6 +5607,222 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56B4C386-9522-4ECE-B788-048FC0CB672A}">
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.6328125" style="43" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="37">
+        <v>5.6576000000000004</v>
+      </c>
+      <c r="B1">
+        <v>3.53</v>
+      </c>
+      <c r="C1" s="36">
+        <f>B1/A1</f>
+        <v>0.623939479638009</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="38">
+        <v>6.35</v>
+      </c>
+      <c r="B2">
+        <v>3.53</v>
+      </c>
+      <c r="C2" s="36">
+        <f>B2/A2</f>
+        <v>0.55590551181102366</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="37">
+        <v>8.1816999999999993</v>
+      </c>
+      <c r="B3">
+        <v>10.67</v>
+      </c>
+      <c r="C3" s="36">
+        <f t="shared" ref="C3:C16" si="0">B3/A3</f>
+        <v>1.3041299485437012</v>
+      </c>
+      <c r="G3" s="36">
+        <f>H3*I3</f>
+        <v>335.60397429943424</v>
+      </c>
+      <c r="H3">
+        <v>23.5</v>
+      </c>
+      <c r="I3" s="44">
+        <f>SUM(C:C)</f>
+        <v>14.281020182954649</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="37">
+        <v>6.8049999999999997</v>
+      </c>
+      <c r="B4">
+        <v>9.06</v>
+      </c>
+      <c r="C4" s="36">
+        <f t="shared" si="0"/>
+        <v>1.3313739897134462</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="39">
+        <v>6.6173000000000002</v>
+      </c>
+      <c r="B5">
+        <v>8.5</v>
+      </c>
+      <c r="C5" s="36">
+        <f t="shared" si="0"/>
+        <v>1.2845118099526998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="37">
+        <v>7.4371</v>
+      </c>
+      <c r="B6">
+        <v>8.18</v>
+      </c>
+      <c r="C6" s="36">
+        <f t="shared" si="0"/>
+        <v>1.0998910865794462</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="37">
+        <v>7.52</v>
+      </c>
+      <c r="B7">
+        <v>11.85</v>
+      </c>
+      <c r="C7" s="36">
+        <f t="shared" si="0"/>
+        <v>1.5757978723404256</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="40">
+        <v>8.6509999999999998</v>
+      </c>
+      <c r="B8">
+        <v>9.4</v>
+      </c>
+      <c r="C8" s="36">
+        <f t="shared" si="0"/>
+        <v>1.0865795861750087</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="41">
+        <v>10.7</v>
+      </c>
+      <c r="B9">
+        <v>9.4</v>
+      </c>
+      <c r="C9" s="36">
+        <f t="shared" si="0"/>
+        <v>0.87850467289719636</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="42">
+        <v>10.5</v>
+      </c>
+      <c r="B10">
+        <v>9.4</v>
+      </c>
+      <c r="C10" s="36">
+        <f t="shared" si="0"/>
+        <v>0.89523809523809528</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="42">
+        <v>12.43</v>
+      </c>
+      <c r="B11">
+        <v>9.4</v>
+      </c>
+      <c r="C11" s="36">
+        <f t="shared" si="0"/>
+        <v>0.75623491552695099</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="37">
+        <v>15.26</v>
+      </c>
+      <c r="B12">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="C12" s="36">
+        <f t="shared" si="0"/>
+        <v>0.60943643512450862</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="37">
+        <v>19.576000000000001</v>
+      </c>
+      <c r="B13">
+        <v>9.4</v>
+      </c>
+      <c r="C13" s="36">
+        <f t="shared" si="0"/>
+        <v>0.48017981201471188</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="38">
+        <v>20.123999999999999</v>
+      </c>
+      <c r="B14">
+        <v>11.33</v>
+      </c>
+      <c r="C14" s="36">
+        <f t="shared" si="0"/>
+        <v>0.56300934207910958</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="37">
+        <v>17.821000000000002</v>
+      </c>
+      <c r="B15">
+        <v>11.33</v>
+      </c>
+      <c r="C15" s="36">
+        <f t="shared" si="0"/>
+        <v>0.63576679198698161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="37">
+        <v>19.2</v>
+      </c>
+      <c r="B16">
+        <v>11.53</v>
+      </c>
+      <c r="C16" s="36">
+        <f t="shared" si="0"/>
+        <v>0.60052083333333328</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BD18CFD-5389-454E-BBF1-4579C4CD4117}">
   <dimension ref="A1:B132"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -6637,7 +6876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2514D165-5F03-4EF1-BE65-CE83882990D5}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -6648,13 +6887,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">

</xml_diff>